<commit_message>
Fix UI sync issues: color hashing, TBD electives, and false UNSATISFIED validations
</commit_message>
<xml_diff>
--- a/DATA/INPUT/phase4_period_assignments.xlsx
+++ b/DATA/INPUT/phase4_period_assignments.xlsx
@@ -449,10 +449,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -497,10 +497,10 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
         <v>0</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -513,10 +513,10 @@
         <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -529,10 +529,10 @@
         <v>3</v>
       </c>
       <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
         <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>